<commit_message>
'morning coffee', 'paneer burger', 'patties paneer', 'pav bhaji', 'tea']
</commit_message>
<xml_diff>
--- a/Menu.xlsx
+++ b/Menu.xlsx
@@ -3,14 +3,11 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="15312" windowHeight="4824" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Chart1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Chart2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Chart3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Menu" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Settings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Menu" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Menu'!$A$1:$G$35</definedName>
@@ -24,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -96,8 +93,15 @@
       <color theme="0"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Cambria"/>
+      <family val="1"/>
+      <b val="1"/>
+      <color theme="0"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -157,6 +161,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -211,7 +221,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -251,15 +261,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
@@ -276,10 +277,30 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -407,624 +428,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="0"/>
-      <spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </title>
-    <plotArea>
-      <layout/>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <varyColors val="0"/>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
-        <gapWidth val="219"/>
-        <overlap val="-27"/>
-        <axId val="574913360"/>
-        <axId val="574918768"/>
-      </barChart>
-      <catAx>
-        <axId val="574913360"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-            <a:round/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </txPr>
-        <crossAx val="574918768"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="0"/>
-      </catAx>
-      <valAx>
-        <axId val="574918768"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </txPr>
-        <crossAx val="574913360"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-      <a:round/>
-    </a:ln>
-  </spPr>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="0"/>
-      <spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </title>
-    <plotArea>
-      <layout/>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <varyColors val="0"/>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
-        <gapWidth val="219"/>
-        <overlap val="-27"/>
-        <axId val="577655936"/>
-        <axId val="577657184"/>
-      </barChart>
-      <catAx>
-        <axId val="577655936"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-            <a:round/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </txPr>
-        <crossAx val="577657184"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="0"/>
-      </catAx>
-      <valAx>
-        <axId val="577657184"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </txPr>
-        <crossAx val="577655936"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-      <a:round/>
-    </a:ln>
-  </spPr>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="0"/>
-      <spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </title>
-    <plotArea>
-      <layout/>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <varyColors val="0"/>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
-        <gapWidth val="219"/>
-        <overlap val="-27"/>
-        <axId val="614990479"/>
-        <axId val="614988815"/>
-      </barChart>
-      <catAx>
-        <axId val="614990479"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:prstDash val="solid"/>
-            <a:round/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </txPr>
-        <crossAx val="614988815"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="0"/>
-      </catAx>
-      <valAx>
-        <axId val="614988815"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-              <a:round/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-            <a:prstDash val="solid"/>
-          </a:ln>
-        </spPr>
-        <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </txPr>
-        <crossAx val="614990479"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-      <a:round/>
-    </a:ln>
-  </spPr>
-</chartSpace>
-</file>
-
-<file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartsheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</chartsheet>
-</file>
-
-<file path=xl/chartsheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartsheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</chartsheet>
-</file>
-
-<file path=xl/chartsheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartsheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</chartsheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <absoluteAnchor>
-    <pos x="0" y="0"/>
-    <ext cx="0" cy="0"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </absoluteAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <absoluteAnchor>
-    <pos x="0" y="0"/>
-    <ext cx="0" cy="0"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </absoluteAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <absoluteAnchor>
-    <pos x="0" y="0"/>
-    <ext cx="0" cy="0"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </absoluteAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1229,18 +632,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="15"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
-    <col width="17.88671875" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
+    <col width="28.44140625" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
     <col width="20.21875" bestFit="1" customWidth="1" style="15" min="3" max="3"/>
-    <col width="20.6640625" bestFit="1" customWidth="1" style="15" min="4" max="4"/>
-    <col width="12.5546875" bestFit="1" customWidth="1" style="28" min="5" max="5"/>
-    <col width="15.77734375" bestFit="1" customWidth="1" style="17" min="6" max="6"/>
-    <col width="14.77734375" bestFit="1" customWidth="1" style="17" min="7" max="7"/>
-    <col width="9.109375" customWidth="1" style="15" min="8" max="8"/>
-    <col width="1.21875" bestFit="1" customWidth="1" style="15" min="9" max="9"/>
+    <col width="23.33203125" bestFit="1" customWidth="1" style="15" min="4" max="4"/>
+    <col width="16.88671875" bestFit="1" customWidth="1" style="33" min="5" max="5"/>
+    <col width="21.44140625" bestFit="1" customWidth="1" style="17" min="6" max="6"/>
+    <col width="23" bestFit="1" customWidth="1" style="17" min="7" max="7"/>
+    <col width="27.44140625" bestFit="1" customWidth="1" style="15" min="8" max="8"/>
+    <col width="24.6640625" customWidth="1" style="15" min="9" max="9"/>
     <col width="9.109375" customWidth="1" style="15" min="10" max="10"/>
     <col width="9.109375" customWidth="1" style="15" min="11" max="16384"/>
   </cols>
@@ -1251,37 +654,37 @@
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="27" t="inlineStr">
         <is>
           <t>Category_Hindi</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="27" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="D1" s="27" t="inlineStr">
         <is>
           <t>Name_Hindi</t>
         </is>
       </c>
-      <c r="E1" s="29" t="inlineStr">
+      <c r="E1" s="34" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="F1" s="19" t="inlineStr">
+      <c r="F1" s="29" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="G1" s="19" t="inlineStr">
+      <c r="G1" s="29" t="inlineStr">
         <is>
           <t>IsMorning</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="27" t="inlineStr">
         <is>
           <t>Image</t>
         </is>
@@ -1290,7 +693,7 @@
     <row r="2" customFormat="1" s="16">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sweet</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1300,16 +703,18 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Gulab Jamun</t>
+          <t>Cold Coffee</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>गुलाब जामुन  (देसी घी)</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>25</v>
+          <t>कोल्ड कॉफ़ी</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1318,19 +723,19 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>images/gulab-jamun.webp</t>
+          <t>images/cold-coffee.webp</t>
         </is>
       </c>
     </row>
     <row r="3" customFormat="1" s="16">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sweet</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1340,16 +745,18 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chocolate Donut</t>
+          <t>Pastry or Pudding</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>चॉकलेट डोनट</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>60</v>
+          <t>पेस्ट्री या पुडिंग</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1363,14 +770,14 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>images/chocolate-donut.webp</t>
+          <t>images/pastry-or-pudding.webp</t>
         </is>
       </c>
     </row>
     <row r="4" customFormat="1" s="16">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sweet</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1388,8 +795,10 @@
           <t>क्रीमरोल</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>40</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1406,7 +815,7 @@
     <row r="5" customFormat="1" s="16">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sweet</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1416,22 +825,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pastry or Pudding</t>
+          <t>Brownie (Walnut)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>पेस्ट्री या पुडिंग</t>
+          <t>ब्राउनी (वालनट)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1441,54 +850,56 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>images/pastry-or-pudding.webp</t>
+          <t>images/brownie-walnut.webp</t>
         </is>
       </c>
     </row>
     <row r="6" customFormat="1" s="16">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sweet</t>
+          <t>Drink</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>मीठा</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Brownie (Walnut)</t>
+          <t>Chocolate Donut</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ब्राउनी (वालनट)</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>60</v>
+          <t>चॉकलेट डोनट</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>images/brownie-walnut.webp</t>
+          <t>images/chocolate-donut.webp</t>
         </is>
       </c>
     </row>
     <row r="7" customFormat="1" s="16">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sweet</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1506,8 +917,10 @@
           <t>मफिन</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>30</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1528,7 +941,7 @@
     <row r="8" customFormat="1" s="16">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Prasad</t>
+          <t>Prasads</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1543,12 +956,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">पेड़ा </t>
+          <t>पेड़ा</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>600</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1570,7 +983,7 @@
     <row r="9" customFormat="1" s="16">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Prasad</t>
+          <t>Prasads</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1612,7 +1025,7 @@
     <row r="10" customFormat="1" s="16">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Prasad</t>
+          <t>Prasads</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1622,7 +1035,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Meva Ladoo </t>
+          <t>Meva Ladoo</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1654,22 +1067,28 @@
     <row r="11" customFormat="1" s="16">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Main</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>मुख्य</t>
+          <t>मीठा</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aaloo Paratha </t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="n">
-        <v>80</v>
+          <t>Aaloo Paratha</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>आलू पराठा</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1678,7 +1097,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1701,15 +1120,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">चाऊमीन </t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>70</v>
+          <t>चाऊमीन</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1744,12 +1165,14 @@
           <t>इडली सांभर</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>80</v>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1763,7 +1186,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="31.05" customFormat="1" customHeight="1" s="16">
+    <row r="14" customFormat="1" s="16">
       <c r="A14" t="inlineStr">
         <is>
           <t>Main</t>
@@ -1784,12 +1207,14 @@
           <t>छोले भटूरे</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>100</v>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1816,7 +1241,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Masala Dosa</t>
+          <t>Masala Dosa</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1824,12 +1249,14 @@
           <t>डोसा</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>120</v>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1864,8 +1291,10 @@
           <t>पिज़्ज़ा</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>250</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1896,7 +1325,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paneer Pizza </t>
+          <t>Paneer Pizza</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1904,8 +1333,10 @@
           <t>पनीर पिज़्ज़ा</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>350</v>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1926,12 +1357,12 @@
     <row r="18" customFormat="1" s="16">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Counter</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>मुख्य</t>
+          <t>मीठा</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1941,11 +1372,13 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">पेटीज - मसाला </t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>40</v>
+          <t>पेटीज - मसाला</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1980,8 +1413,10 @@
           <t>फ्रेंच फ्राइज</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>100</v>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -2020,8 +1455,10 @@
           <t>बर्गर</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>70</v>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -2060,8 +1497,10 @@
           <t>कॉफ़ी</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>30</v>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -2070,7 +1509,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -2078,26 +1517,28 @@
     <row r="22" customFormat="1" s="16">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Drink</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>पेय</t>
+          <t>मीठा</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cold Coffee</t>
+          <t>Gulab Jamun</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>कोल्ड कॉफ़ी</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>80</v>
+          <t>गुलाब जामुन  (देसी घी)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -2106,24 +1547,24 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>images/cold-coffee.webp</t>
+          <t>images/gulab-jamun.webp</t>
         </is>
       </c>
     </row>
     <row r="23" customFormat="1" s="16">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Drink</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>पेय</t>
+          <t>मीठा</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2133,11 +1574,13 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">चाय </t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>20</v>
+          <t>चाय</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -2158,12 +1601,12 @@
     <row r="24" customFormat="1" s="16">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Drink</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>पेय</t>
+          <t>मीठा</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2173,11 +1616,13 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">जल </t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>20</v>
+          <t>जल</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -2216,20 +1661,26 @@
           <t>मैंगो  ड्रिंक</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v>20</v>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>images/mango-drink.webp</t>
+        </is>
+      </c>
     </row>
     <row r="26" customFormat="1" s="16">
       <c r="A26" t="inlineStr">
@@ -2252,17 +1703,19 @@
           <t>लस्सी</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>60</v>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -2280,7 +1733,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lemon Soda </t>
+          <t>Lemon Soda</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2288,30 +1741,32 @@
           <t>सोडा</t>
         </is>
       </c>
-      <c r="E27" t="n">
-        <v>30</v>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
     </row>
-    <row r="28" ht="31.05" customFormat="1" customHeight="1" s="16">
+    <row r="28" customFormat="1" s="16">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Counter</t>
+          <t>Drink</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>काउन्टर</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2324,8 +1779,10 @@
           <t>छोले कुलचे</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>70</v>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -2346,17 +1803,17 @@
     <row r="29" customFormat="1" s="16">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Counter</t>
+          <t>Drink</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>काउन्टर</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patties Paneer </t>
+          <t>Patties Paneer</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2364,8 +1821,10 @@
           <t>पटीज़ - पनीर</t>
         </is>
       </c>
-      <c r="E29" t="n">
-        <v>60</v>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -2382,12 +1841,12 @@
     <row r="30" customFormat="1" s="16">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Counter</t>
+          <t>Drink</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>काउन्टर</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2400,8 +1859,10 @@
           <t>सैंडविच (ग्रिल्ड)</t>
         </is>
       </c>
-      <c r="E30" t="n">
-        <v>70</v>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -2419,15 +1880,15 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="31.05" customFormat="1" customHeight="1" s="16">
+    <row r="31" customFormat="1" s="16">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Counter</t>
+          <t>Sweetiya</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>काउन्टर</t>
+          <t>मीठा</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2440,8 +1901,10 @@
           <t>समोसा</t>
         </is>
       </c>
-      <c r="E31" t="n">
-        <v>20</v>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -2462,12 +1925,12 @@
     <row r="32" customFormat="1" s="16">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Chaat</t>
+          <t>Drink</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>चाट</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2480,8 +1943,10 @@
           <t>आलू टिक्की चाट</t>
         </is>
       </c>
-      <c r="E32" t="n">
-        <v>60</v>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -2502,12 +1967,12 @@
     <row r="33" customFormat="1" s="16">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Counter</t>
+          <t>Drink</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>चाट</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2520,8 +1985,10 @@
           <t>पाव भाजी</t>
         </is>
       </c>
-      <c r="E33" t="n">
-        <v>80</v>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -2538,12 +2005,12 @@
     <row r="34" customFormat="1" s="16">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Chaat</t>
+          <t>Prasads</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>चाट</t>
+          <t>प्रसाद</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2556,12 +2023,14 @@
           <t>समोसा छोला</t>
         </is>
       </c>
-      <c r="E34" t="n">
-        <v>60</v>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2578,12 +2047,12 @@
     <row r="35" customFormat="1" s="16">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Counter</t>
+          <t>Drink</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>चाट</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2596,8 +2065,10 @@
           <t>समोसा मटर</t>
         </is>
       </c>
-      <c r="E35" t="n">
-        <v>60</v>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -2639,12 +2110,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
@@ -2652,10 +2123,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Counter</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
+          <t>Drink</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>पेय</t>
+        </is>
+      </c>
       <c r="C37" t="inlineStr">
         <is>
           <t>Paneer Burger</t>
@@ -2682,24 +2157,6 @@
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G35">
@@ -2722,10 +2179,10 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5546875" defaultRowHeight="15.6"/>
   <cols>
     <col width="37.77734375" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
-    <col width="48.77734375" bestFit="1" customWidth="1" style="23" min="2" max="2"/>
-    <col width="53.21875" customWidth="1" style="24" min="3" max="3"/>
-    <col width="12.5546875" customWidth="1" style="24" min="4" max="4"/>
-    <col width="12.5546875" customWidth="1" style="24" min="5" max="16384"/>
+    <col width="48.77734375" bestFit="1" customWidth="1" style="20" min="2" max="2"/>
+    <col width="53.21875" customWidth="1" style="21" min="3" max="3"/>
+    <col width="12.5546875" customWidth="1" style="21" min="4" max="5"/>
+    <col width="12.5546875" customWidth="1" style="21" min="6" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2746,7 +2203,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>⚙️  GENERAL</t>
         </is>
@@ -2802,7 +2259,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>🌅  MORNING MENU</t>
         </is>
@@ -2839,7 +2296,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>🔤  TYPOGRAPHY</t>
         </is>
@@ -3096,7 +2553,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="25" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>📐  SPACING</t>
         </is>

</xml_diff>

<commit_message>
'evening of august 15'
</commit_message>
<xml_diff>
--- a/Menu.xlsx
+++ b/Menu.xlsx
@@ -632,7 +632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="15"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
@@ -689,6 +689,11 @@
           <t>Image</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Featured</t>
+        </is>
+      </c>
     </row>
     <row r="2" customFormat="1" s="16">
       <c r="A2" t="inlineStr">
@@ -703,17 +708,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cold Coffee</t>
+          <t>Cream Roll</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>कोल्ड कॉफ़ी</t>
+          <t>क्रीमरोल</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -723,12 +728,13 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>images/cold-coffee.webp</t>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -745,17 +751,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cream Roll</t>
+          <t>Gulab Jamun</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>क्रीमरोल</t>
+          <t>गुलाब जामुन  (देसी घी)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>25</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -768,32 +774,41 @@
           <t>true</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>images/gulab-jamun.webp</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
     </row>
     <row r="4" customFormat="1" s="16">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sweet</t>
+          <t>Prasad</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>मीठा</t>
+          <t>प्रसाद</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chocolate Donut</t>
+          <t>Besan Ladoo</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>चॉकलेट डोनट</t>
+          <t>बेसन लड्डू  (देसी घी)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>500</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -808,34 +823,39 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>images/chocolate-donut.webp</t>
+          <t>images/besan-ladoo.webp</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="5" customFormat="1" s="16">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sweet</t>
+          <t>Prasad</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>मीठा</t>
+          <t>प्रसाद</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Brownie (Walnut)</t>
+          <t>Peda</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ब्राउनी (वालनट)</t>
+          <t>पेड़ा</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>600</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -850,7 +870,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>images/brownie-walnut.webp</t>
+          <t>images/peda-2.webp</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -867,17 +892,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Gulab Jamun</t>
+          <t>Chocolate Donut</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>गुलाब जामुन  (देसी घी)</t>
+          <t>चॉकलेट डोनट</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -892,34 +917,39 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>images/gulab-jamun.webp</t>
+          <t>images/chocolate-donut.webp</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="7" customFormat="1" s="16">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Prasad</t>
+          <t>Sweet</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>प्रसाद</t>
+          <t>मीठा</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Besan Ladoo</t>
+          <t>Brownie (Walnut)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>बेसन लड्डू  (देसी घी)</t>
+          <t>ब्राउनी (वालनट)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -934,34 +964,39 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>images/besan-ladoo.webp</t>
+          <t>images/brownie-walnut.webp</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="8" customFormat="1" s="16">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Prasad</t>
+          <t>Sweet</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>प्रसाद</t>
+          <t>मीठा</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Peda</t>
+          <t>Muffin</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>पेड़ा</t>
+          <t>मफिन</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -976,34 +1011,39 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>images/peda-2.webp</t>
+          <t>images/muffin.webp</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="9" customFormat="1" s="16">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sweet</t>
+          <t>Main</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>मीठा</t>
+          <t>मुख्य</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Muffin</t>
+          <t>Chowmein</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>मफिन</t>
+          <t>चाऊमीन</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>70</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1013,12 +1053,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>images/muffin.webp</t>
+          <t>images/chowmein.webp</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -1035,17 +1080,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Masala Dosa</t>
+          <t>Idli Sambhar</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>डोसा</t>
+          <t>इडली सांभर</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>80</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1060,34 +1105,39 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>images/masala-dosa.webp</t>
+          <t>images/idli-sambhar.webp</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="11" customFormat="1" s="16">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Main</t>
+          <t>Sweet</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>मुख्य</t>
+          <t>मीठा</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chole Bhature</t>
+          <t>Pastry or Pudding</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>छोले भटूरे</t>
+          <t>पेस्ट्री या पुडिंग</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>63</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1097,12 +1147,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>images/chole-bhature.webp</t>
+          <t>images/pastry-or-pudding.webp</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -1119,17 +1174,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Chowmein</t>
+          <t>Masala Dosa</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>चाऊमीन</t>
+          <t>डोसा</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>120</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1144,7 +1199,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>images/chowmein.webp</t>
+          <t>images/masala-dosa.webp</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -1161,17 +1221,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Idli Sambhar</t>
+          <t>Paneer Burger</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>इडली सांभर</t>
+          <t>पनीर बर्गर</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>120</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1186,34 +1246,39 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>images/idli-sambhar.webp</t>
+          <t>images/paneer-burger.webp</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="14" customFormat="1" s="16">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Main</t>
+          <t>Drinks</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>मुख्य</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>French Fries</t>
+          <t>Coffee</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>फ्रेंच फ्राइज</t>
+          <t>कॉफ़ी</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1223,39 +1288,44 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>images/french-fries.webp</t>
+          <t>images/coffee.webp</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="15" customFormat="1" s="16">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Main</t>
+          <t>Drinks</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>मुख्य</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pizza</t>
+          <t>Lassi</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>पिज़्ज़ा</t>
+          <t>लस्सी</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1265,39 +1335,40 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>images/pizza.webp</t>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="16" customFormat="1" s="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Main</t>
+          <t>Drinks</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>मुख्य</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Paneer Pizza</t>
+          <t>Lemon Soda</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>पनीर पिज़्ज़ा</t>
+          <t>सोडा</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>30</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1307,39 +1378,40 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>images/paneer-pizza.webp</t>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="17" customFormat="1" s="16">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sweet</t>
+          <t>Drinks</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>मीठा</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pastry or Pudding</t>
+          <t>Mango  Drink</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>पेस्ट्री या पुडिंग</t>
+          <t>मैंगो  ड्रिंक</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1354,34 +1426,39 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>images/pastry-or-pudding.webp</t>
+          <t>images/mango-drink.webp</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="18" customFormat="1" s="16">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Main</t>
+          <t>Drinks</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>मुख्य</t>
+          <t>पेय</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Burger</t>
+          <t>Orange Drink</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>बर्गर</t>
+          <t>ऑरेंज ड्रिंक</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1391,12 +1468,13 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>images/burger.webp</t>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -1413,12 +1491,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Tea</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>जल</t>
+          <t>चाय</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1438,34 +1516,39 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>images/water.webp</t>
+          <t>images/tea-2.webp</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="20" customFormat="1" s="16">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Drinks</t>
+          <t>Main</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>पेय</t>
+          <t>मुख्य</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tea</t>
+          <t>Paneer Pizza</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>चाय</t>
+          <t>पनीर पिज़्ज़ा</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>350</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1475,12 +1558,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>images/tea-2.webp</t>
+          <t>images/paneer-pizza.webp</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -1497,17 +1585,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Coffee</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>कॉफ़ी</t>
+          <t>जल</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1522,7 +1610,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>images/coffee.webp</t>
+          <t>images/water.webp</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -1539,17 +1632,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Lassi</t>
+          <t>Cold Coffee</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>लस्सी</t>
+          <t>कोल्ड कॉफ़ी</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>80</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1559,35 +1652,44 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>images/cold-coffee.webp</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
     </row>
     <row r="23" customFormat="1" s="16">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Drinks</t>
+          <t>Chaat Paat</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>पेय</t>
+          <t>चट पट</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mango  Drink</t>
+          <t>Chole Kulche</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>मैंगो  ड्रिंक</t>
+          <t>छोले कुलचे</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>70</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1602,34 +1704,39 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>images/mango-drink.webp</t>
+          <t>images/chole-kulche.webp</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="24" customFormat="1" s="16">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Drinks</t>
+          <t>Chaat Paat</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>पेय</t>
+          <t>चट पट</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Orange Drink</t>
+          <t>Pav bhaji</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ऑरेंज ड्रिंक</t>
+          <t>पाव भाजी</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>80</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1639,35 +1746,44 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>images/pav-bhaji.webp</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="25" customFormat="1" s="16">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Main</t>
+          <t>Chaat Paat</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>मुख्य</t>
+          <t>चट पट</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Paneer Burger</t>
+          <t>Tikki Chaat</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>पनीर बर्गर</t>
+          <t>आलू टिक्की चाट</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1677,39 +1793,44 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>images/paneer-burger.webp</t>
+          <t>images/tikki-chaat.webp</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="26" customFormat="1" s="16">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Drinks</t>
+          <t>Chaat Paat</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>पेय</t>
+          <t>चट पट</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Lemon Soda</t>
+          <t>Samosa</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>सोडा</t>
+          <t>समोसा</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>20</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1722,7 +1843,16 @@
           <t>true</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>images/samosa.webp</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="27" customFormat="1" s="16">
       <c r="A27" t="inlineStr">
@@ -1737,17 +1867,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Samosa</t>
+          <t>Samosa Matar</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>समोसा</t>
+          <t>समोसा मटर</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1757,12 +1887,13 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>images/samosa.webp</t>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
@@ -1779,17 +1910,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Samosa Matar</t>
+          <t>Patties - Masala</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>समोसा मटर</t>
+          <t>पेटीज - मसाला</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1799,10 +1930,15 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="29" customFormat="1" s="16">
       <c r="A29" t="inlineStr">
@@ -1845,6 +1981,11 @@
           <t>images/samosa-chhola.webp</t>
         </is>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="30" customFormat="1" s="16">
       <c r="A30" t="inlineStr">
@@ -1859,17 +2000,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Chole Kulche</t>
+          <t>Patties Paneer</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>छोले कुलचे</t>
+          <t>पटीज़ - पनीर</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>60</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1879,39 +2020,44 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>images/chole-kulche.webp</t>
+          <t>images/patties-paneer.webp</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="31" customFormat="1" s="16">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Chaat Paat</t>
+          <t>Prasad</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>चट पट</t>
+          <t>प्रसाद</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Pav bhaji</t>
+          <t>Meva Ladoo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>पाव भाजी</t>
+          <t>मेवा लड्डू (देसी घी)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>800</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1921,39 +2067,44 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>images/pav-bhaji.webp</t>
+          <t>images/meva-ladoo.webp</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="32" customFormat="1" s="16">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Chaat Paat</t>
+          <t>Main</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>चट पट</t>
+          <t>मुख्य</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tikki Chaat</t>
+          <t>Pizza</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>आलू टिक्की चाट</t>
+          <t>पिज़्ज़ा</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>250</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1963,39 +2114,44 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>images/tikki-chaat.webp</t>
+          <t>images/pizza.webp</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="33" customFormat="1" s="16">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Chaat Paat</t>
+          <t>Main</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>चट पट</t>
+          <t>मुख्य</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Patties - Masala</t>
+          <t>French Fries</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>पेटीज - मसाला</t>
+          <t>फ्रेंच फ्राइज</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>100</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2005,35 +2161,44 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>images/french-fries.webp</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
     </row>
     <row r="34" customFormat="1" s="16">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Chaat Paat</t>
+          <t>Main</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>चट पट</t>
+          <t>मुख्य</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Patties Paneer</t>
+          <t>Chole Bhature</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>पटीज़ - पनीर</t>
+          <t>छोले भटूरे</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>100</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2048,34 +2213,39 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>images/patties-paneer.webp</t>
+          <t>images/chole-bhature.webp</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="35" customFormat="1" s="16">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Prasad</t>
+          <t>Main</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>प्रसाद</t>
+          <t>मुख्य</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Meva Ladoo</t>
+          <t>Burger</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>मेवा लड्डू (देसी घी)</t>
+          <t>बर्गर</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>70</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2085,12 +2255,17 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>images/meva-ladoo.webp</t>
+          <t>images/burger.webp</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
@@ -2133,6 +2308,11 @@
       <c r="H36" t="inlineStr">
         <is>
           <t>images/sandwich.webp</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>

</xml_diff>